<commit_message>
Simple Flow: record shortcut principle + reclassify findings + trim Milos round-2
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/OpenQuestions-for-Milos-Round2.xlsx
+++ b/build/simple-flow/OpenQuestions-for-Milos-Round2.xlsx
@@ -33,10 +33,11 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F4E78"/>
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +47,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F5FA"/>
       </patternFill>
     </fill>
   </fills>
@@ -59,31 +65,45 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D7E2"/>
       </left>
       <right style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D7E2"/>
       </right>
       <top style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D7E2"/>
       </top>
       <bottom style="thin">
-        <color rgb="00BFBFBF"/>
+        <color rgb="00D0D7E2"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -449,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -461,7 +481,7 @@
     <col width="30" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>#</t>
@@ -479,7 +499,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Question (plain, self-contained, with a concrete example where helpful)</t>
+          <t>Question</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -502,218 +522,156 @@
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Round-1 Q7</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Mark-Reviewed dialog — review note field</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>The Mark Reviewed dialog captures only the vehicle identification number (VIN); there is no optional "review note" field. Is that intended for v1 (so we will set the expectation to "no note field"), or is the missing note field a bug to be fixed? Example: today a reviewer signs off by entering the VIN and confirming — there is nowhere to type a free-text note about the review.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Determines whether we write the expected result as "no note field" (intended) or leave the case failing against a bug. We do not want to lock in the wrong expectation.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Mark-Reviewed dialog - review note field</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>The Mark Reviewed dialog captures only the vehicle identification number (VIN); there is no optional 'review note' field. We are treating this as an intended Simple Mode simplification (so we will set the expectation to 'no note field') - can you confirm that is correct for v1, or do you want the optional note field added back? Example: today a reviewer signs off by entering the VIN and confirming - there is nowhere to type a free-text note about the review.</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Just a quick confirmation so we lock in the right expectation. We assume 'no note field' (intended simplification) unless you say otherwise.</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>SF-REV-10</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Round-1 Q8</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Review → Reviewed → Complete state machine</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>After a reviewer clicks "Mark Reviewed", should the work order move to a distinct "Reviewed" state before it becomes "Complete", or should it go straight from Review to Complete? Today it jumps straight to Complete with no separate "Reviewed" state in between. Example: reviewer opens a work order that was sent to review, clicks Mark Reviewed → we expected a green "Reviewed / sign-off complete" holding state and then a separate final "Complete Work Order" action, but instead the order becomes Complete in one step.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Decides the review state-machine expectations and the "invoicing blocked until reviewed" checks. (This may be intended admin auto-progression — please confirm.)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>SF-REV-08, SF-REV-11</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Round-1 Q9</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Tech-story entry points (Story 17 vs older wording)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Does Story 17 (tech story captured via the completion modal at completion plus inline on the line) fully supersede the older 'tech story lives on the line only' behavior (S15-R2)? Please confirm the authoritative tech-story entry points for v1. Example: our live testing showed the completion modal gate for the tech story working, so we believe Story 17 is current - we just need your explicit confirmation.</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Confirms whether the tech-story gate-modal cases are authoritative, or whether we should revert to line-only behavior.</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>SF-TECH-*</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Round-1 Q9</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Tech-story entry points (Story 17 vs older wording)</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Does Story 17 (tech story captured via the completion modal at completion plus inline on the line) fully supersede the older "tech story lives on the line only" behavior (S15-R2)? Please confirm the authoritative tech-story entry points for v1. Example: our live testing showed the completion modal gate for the tech story working, so we believe Story 17 is current — we just need your explicit confirmation.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Confirms whether the tech-story gate-modal cases are authoritative, or whether we should revert to line-only behavior.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>SF-TECH-*</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Round-1 Q2</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Inventory lifecycle on completion (data-integrity)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>With the No-PO / skip path removed and a purchase order always created, when a work order is completed do in-stock / inventory parts still decrement on-hand inventory and post to Part History at completion (i.e., the real part lifecycle still runs)? Example: a work order uses 2 units of a part already in stock; on completion we expect on-hand to drop by 2 and a Part History movement to be recorded.</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>This is a data-integrity invariant. Your Round-1 answer confirmed the No-PO path is removed but did not explicitly confirm that normal completion still moves inventory and writes history. (Under our shortcut rule, a faster completion is fine - but only if inventory and Part History stay correct.)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>SF-COMP-07, SF-QB-01</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>Round-1 Q2</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Inventory lifecycle on completion</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>With the No-PO / skip path removed and a purchase order always created, when a work order is completed do in-stock / inventory parts still decrement on-hand inventory and post to Part History at completion (i.e., the real part lifecycle still runs)? Example: a work order uses 2 units of a part already in stock; on completion we expect on-hand to drop by 2 and a Part History movement to be recorded.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>This is a data-integrity invariant. Your Round-1 answer confirmed the No-PO path is removed but did not explicitly confirm that normal completion still moves inventory and writes history.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>SF-COMP-07, SF-QB-01</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr"/>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>New (BUG-9)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>'New Part Request' required fields (Category / Sell Price)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>The vendorless 'New Part Request' sub-form currently requires a Category, but spec S5-R1 lists only description + quantity + sell price. Is requiring a Category intended for v1 (so we add 'Category required' to the expected result), or is it a bug? And, separately, should Sell Price be a required field? Example: today, entering only description + quantity + sell price does not save - the form blocks with 'Category is a required field'; meanwhile Sell Price is not enforced as required at all.</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Determines the correct required-field set for the part-request cases; the spec and the build currently disagree in both directions (Category is required but not in spec; Sell Price is in spec but not enforced). Note: this is an ADDED required field, not a skipped step, so it is not covered by the Simple Mode shortcut rule.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>SF-VPART-01, SF-VPART-02</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>New (BUG-9)</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>"New Part Request" required fields (Category / Sell Price)</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>The vendorless "New Part Request" sub-form currently requires a Category, but spec S5-R1 lists only description + quantity + sell price. Is requiring a Category intended for v1 (so we add "Category required" to the expected result), or is it a bug? And, separately, should Sell Price be a required field? Example: today, entering only description + quantity + sell price does not save — the form blocks with "Category is a required field"; meanwhile Sell Price is not enforced as required at all.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Determines the correct required-field set for the part-request cases; the spec and the build currently disagree in both directions (Category is required but not in spec; Sell Price is in spec but not enforced).</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>SF-VPART-01, SF-VPART-02</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>New (BUG-10)</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Resolve Cores — wizard step vs line-level</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>For a cored part on a work order, the completion wizard has no distinct "Resolve Cores" step — core OK / Not-OK is handled at the line level and completion goes Details → Success. Is this the intended v1 behavior, or should there be a dedicated Resolve-Cores step in the completion wizard? Example: a cored part generates a "Core" sub-line on the work order with Ok / Not Ok controls on the line's Parts view, but when completing the work order the wizard shows only Details then Success — no core-resolution step with a running "+$ to invoice" total.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Decides whether the core-resolution cases expect a wizard step or a line-level control — they are written today to expect a wizard step.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>SF-CORE-01..10</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>New (SF-PERM-06 / BUG-6 / BUG-7)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Backend enforcement of completion / review-sign-off permissions</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>We found that the backend does not enforce the completion / review-sign-off permission atoms — a user without the permission (e.g. a Technician) can complete a work order or sign off a review directly via the API; only the UI hides the buttons. Is this intended (front-end-only gating, consistent with the Work-Order Create-&amp;-Edit atom-collapse in SV-7864), or should the backend enforce these permissions? Example: a Technician who cannot see the "Complete Work Order" button in the UI can still call the completion endpoint and the work order completes successfully (HTTP 201) instead of being rejected (HTTP 403).</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Decides whether the permission cases pass (FE-only gating is acceptable) or fail (a backend enforcement gap). This resolves the SV-8183 "backend enforces the atoms" vs SV-7864 "atom-collapse" contradiction.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>We found that the backend does not enforce the completion / review-sign-off permission atoms - a user without the permission (e.g. a Technician) can complete a work order or sign off a review directly via the API; only the UI hides the buttons. Is this intended (front-end-only gating, consistent with the Work-Order Create-&amp;-Edit atom-collapse in SV-7864), or should the backend enforce these permissions? Example: a Technician who cannot see the 'Complete Work Order' button in the UI can still call the completion endpoint and the work order completes successfully (HTTP 201) instead of being rejected (HTTP 403).</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Decides whether the permission cases pass (FE-only gating is acceptable) or fail (a backend enforcement gap). This resolves the SV-8183 'backend enforces the atoms' vs SV-7864 'atom-collapse' contradiction. This is an enforcement question, not a flow-skip.</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
         <is>
           <t>SF-PERM-06</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr"/>
+      <c r="G6" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -726,76 +684,97 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Open Questions for Milos — Round 2</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" s="7" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Feature: Simple Mode / Streamlined Work Order Completion &amp; Receiving (Epic SV-7301)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Raised by: ShopView QA</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>For: Milos Vasic (Product Owner / spec author)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
+      <c r="A6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>These are QA's remaining open items after Round 1 — the items left unanswered or</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ambiguous, plus new findings that were not on the first sheet. Each question is</t>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>ambiguous, plus new findings that were not on the first sheet. Two earlier items</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>(the 'distinct Reviewed state' and the 'Resolve-Cores wizard step') have been</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>withdrawn: they are now treated as expected Simple Mode shortcuts (each reaches</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>the same end state faster with no error or data loss). Each question is</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>self-contained (with a concrete example where it helps); no access to the QA test</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>repository is needed to answer. Please add your answer in the last column of the</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>'Open Questions R2' tab for each row.</t>
         </is>

</xml_diff>